<commit_message>
Correccion metodologica integral: ajuste NUTS real, modelo BYM2, tablas empiricas y eliminacion de datos simulados
</commit_message>
<xml_diff>
--- a/outputs/data/reporte_calidad.xlsx
+++ b/outputs/data/reporte_calidad.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Métrica</t>
   </si>
@@ -22,7 +22,7 @@
     <t>Valor</t>
   </si>
   <si>
-    <t>Registros Iniciales</t>
+    <t>Registros Iniciales (Excel crudo)</t>
   </si>
   <si>
     <t>Duplicados Eliminados</t>
@@ -34,19 +34,43 @@
     <t>Coordenadas Fuera de Bounding Box Eliminadas</t>
   </si>
   <si>
-    <t>Registros Limpios Finales</t>
-  </si>
-  <si>
-    <t>Valores Faltantes en Edad</t>
-  </si>
-  <si>
-    <t>Valores Faltantes en Arma</t>
-  </si>
-  <si>
-    <t>Valores Faltantes en Presunto Móvil</t>
-  </si>
-  <si>
-    <t>Valores Faltantes en Antecedentes</t>
+    <t>Registros Limpios Finales (N total)</t>
+  </si>
+  <si>
+    <t>Valores Faltantes en Edad (NaN)</t>
+  </si>
+  <si>
+    <t>Valores Válidos en Edad (n reportado)</t>
+  </si>
+  <si>
+    <t>Valores Faltantes en Antecedentes (100% - Excluido)</t>
+  </si>
+  <si>
+    <t>Eventos sin Subcircuito (post-cruce)</t>
+  </si>
+  <si>
+    <t>Víctimas Hombres</t>
+  </si>
+  <si>
+    <t>Víctimas Mujeres</t>
+  </si>
+  <si>
+    <t>Víctimas No Determinadas</t>
+  </si>
+  <si>
+    <t>Total Suma Sexo (Control)</t>
+  </si>
+  <si>
+    <t>Homicidios Año 2024 (Año completo)</t>
+  </si>
+  <si>
+    <t>Homicidios Año 2025 (Año completo)</t>
+  </si>
+  <si>
+    <t>Homicidios Año 2026 (Solo Enero)</t>
+  </si>
+  <si>
+    <t>Total Suma Temporal (Control)</t>
   </si>
 </sst>
 </file>
@@ -404,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -468,7 +492,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>4402</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -476,7 +500,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>4634</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -484,6 +508,70 @@
         <v>10</v>
       </c>
       <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>4227</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>4634</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>1926</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>2506</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
         <v>4634</v>
       </c>
     </row>

</xml_diff>